<commit_message>
etapa 3 avanzando, falta seguir ajustando
</commit_message>
<xml_diff>
--- a/output/_temp/etapa_1_limpieza_base/Cierre de OT Turno 02.04 al 08.04.xlsx
+++ b/output/_temp/etapa_1_limpieza_base/Cierre de OT Turno 02.04 al 08.04.xlsx
@@ -827,7 +827,11 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n"/>
-      <c r="L6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">

</xml_diff>